<commit_message>
fix: improve dataset & some minor problem, add new search feature in detail event
</commit_message>
<xml_diff>
--- a/data_clean/data_merged.xlsx
+++ b/data_clean/data_merged.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Documents\All Work Files\1. PE New Report\data_clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A152BA-22EA-484A-A22F-9661A003C24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1589DE59-18C2-40E3-9430-03B80D580DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3548,7 +3548,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -3587,9 +3587,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -3601,15 +3599,61 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -3620,6 +3664,40 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F38F7656-86CA-4821-ADA1-5488F5CEC9A1}" name="Table1" displayName="Table1" ref="A1:Y314" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3">
+  <autoFilter ref="A1:Y314" xr:uid="{F38F7656-86CA-4821-ADA1-5488F5CEC9A1}"/>
+  <tableColumns count="25">
+    <tableColumn id="1" xr3:uid="{039698E2-019D-4AFA-8ACB-10939541A822}" name="Email"/>
+    <tableColumn id="2" xr3:uid="{F0B53F50-E27A-4C90-AA9D-A84B1E0DB011}" name="Nama"/>
+    <tableColumn id="3" xr3:uid="{A8718DD6-247B-4B12-B9ED-02413F488A3F}" name="No WhatsApp"/>
+    <tableColumn id="4" xr3:uid="{002BD4EC-270A-41BE-89D6-EEC30CD8EBBE}" name="Kota - Provinsi"/>
+    <tableColumn id="5" xr3:uid="{9AF223A0-30B9-412E-BD34-0749345E1DC5}" name="Tempat Kegiatan"/>
+    <tableColumn id="6" xr3:uid="{B965C319-E859-4E80-ADCE-D9D868EE3DF4}" name="Tanggal" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{0764D467-1E41-4062-8E3F-57ABBC25DEFF}" name="Sesi"/>
+    <tableColumn id="8" xr3:uid="{48B11DBE-00E1-4C18-9924-E853A00EE4EE}" name="Jumlah Sesi"/>
+    <tableColumn id="9" xr3:uid="{2036A2E3-9C96-4DF7-B233-DE478FEFB31C}" name="Tahun"/>
+    <tableColumn id="10" xr3:uid="{4011E0EC-0619-4904-BD0B-1F81E701860D}" name="Bulan"/>
+    <tableColumn id="11" xr3:uid="{CF821166-36F2-4E60-935C-7243AF8FFB7A}" name="Kategori"/>
+    <tableColumn id="12" xr3:uid="{3E8AAF3D-314E-4163-80BE-4B8128C65FBC}" name="Nama Event"/>
+    <tableColumn id="13" xr3:uid="{421CFBC9-4A8C-457C-8A2E-48541C4D2F52}" name="Lokasi Event"/>
+    <tableColumn id="14" xr3:uid="{7D76B757-FD8E-492E-8808-D6DD7A2F4960}" name="Gender"/>
+    <tableColumn id="15" xr3:uid="{82C967A4-9796-44F3-9C18-48AB06C138CC}" name="Kota"/>
+    <tableColumn id="16" xr3:uid="{7B5DD4E8-61EB-443E-9AA5-CE3C5C9DD53D}" name="Provinsi"/>
+    <tableColumn id="17" xr3:uid="{4771CA65-6E51-4436-802D-284D20111AE7}" name="Usia"/>
+    <tableColumn id="18" xr3:uid="{2B7692F7-6692-4662-B210-8342ACB84741}" name="Kelompok Usia"/>
+    <tableColumn id="19" xr3:uid="{3EBFD3FE-8AA6-4F32-B6BC-D5CA2B1141FB}" name="Profesi (Asli)"/>
+    <tableColumn id="20" xr3:uid="{1D3B455E-FDC7-45A5-9B0B-89232ABBA013}" name="Kategori Profesi"/>
+    <tableColumn id="21" xr3:uid="{90BA8C37-E4C3-4FD0-813B-7AA8C7023455}" name="Harapan (Asli)"/>
+    <tableColumn id="22" xr3:uid="{02FA6104-8D44-4757-8BB5-203B4AED2B4D}" name="Topik Harapan"/>
+    <tableColumn id="23" xr3:uid="{41A5D24A-2F9C-43B9-9DCE-26AA34BBD6B4}" name="Keluhan (Asli)"/>
+    <tableColumn id="24" xr3:uid="{1D70B43B-886D-4226-B4BB-0D2D55DC4290}" name="Topik Keluhan"/>
+    <tableColumn id="25" xr3:uid="{6E684841-431B-4E90-BFE4-93684C9B6CFF}" name="Wilayah"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3909,81 +3987,101 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y314"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.90625" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" customWidth="1"/>
+    <col min="8" max="8" width="12.36328125" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" customWidth="1"/>
+    <col min="12" max="12" width="12.90625" customWidth="1"/>
+    <col min="13" max="13" width="13.1796875" customWidth="1"/>
+    <col min="14" max="14" width="9" customWidth="1"/>
+    <col min="16" max="16" width="9.453125" customWidth="1"/>
+    <col min="18" max="18" width="15.26953125" customWidth="1"/>
+    <col min="19" max="19" width="13.26953125" customWidth="1"/>
+    <col min="20" max="20" width="16.08984375" customWidth="1"/>
+    <col min="21" max="21" width="14.6328125" customWidth="1"/>
+    <col min="22" max="22" width="15.08984375" customWidth="1"/>
+    <col min="23" max="23" width="14.26953125" customWidth="1"/>
+    <col min="24" max="24" width="14.7265625" customWidth="1"/>
+    <col min="25" max="25" width="9.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -4003,7 +4101,7 @@
       <c r="E2" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="1">
         <v>45515</v>
       </c>
       <c r="G2" t="s">
@@ -4056,7 +4154,7 @@
       <c r="E3" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>45515</v>
       </c>
       <c r="G3" t="s">
@@ -4109,7 +4207,7 @@
       <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>45515</v>
       </c>
       <c r="G4" t="s">
@@ -4162,7 +4260,7 @@
       <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>45515</v>
       </c>
       <c r="G5" t="s">
@@ -4215,7 +4313,7 @@
       <c r="E6" t="s">
         <v>29</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="1">
         <v>45515</v>
       </c>
       <c r="G6" t="s">
@@ -4268,7 +4366,7 @@
       <c r="E7" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>45515</v>
       </c>
       <c r="G7" t="s">
@@ -4321,7 +4419,7 @@
       <c r="E8" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>45515</v>
       </c>
       <c r="G8" t="s">
@@ -4374,7 +4472,7 @@
       <c r="E9" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>45515</v>
       </c>
       <c r="G9" t="s">
@@ -4427,7 +4525,7 @@
       <c r="E10" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>45515</v>
       </c>
       <c r="G10" t="s">
@@ -4480,7 +4578,7 @@
       <c r="E11" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>45515</v>
       </c>
       <c r="G11" t="s">
@@ -4533,7 +4631,7 @@
       <c r="E12" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="1">
         <v>45515</v>
       </c>
       <c r="G12" t="s">
@@ -4586,7 +4684,7 @@
       <c r="E13" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="1">
         <v>45515</v>
       </c>
       <c r="G13" t="s">
@@ -4639,7 +4737,7 @@
       <c r="E14" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="1">
         <v>45515</v>
       </c>
       <c r="G14" t="s">
@@ -4692,7 +4790,7 @@
       <c r="E15" t="s">
         <v>29</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="1">
         <v>45515</v>
       </c>
       <c r="G15" t="s">
@@ -4745,7 +4843,7 @@
       <c r="E16" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>45515</v>
       </c>
       <c r="G16" t="s">
@@ -4798,7 +4896,7 @@
       <c r="E17" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>45515</v>
       </c>
       <c r="G17" t="s">
@@ -4851,7 +4949,7 @@
       <c r="E18" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="1">
         <v>45515</v>
       </c>
       <c r="G18" t="s">
@@ -4904,7 +5002,7 @@
       <c r="E19" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19" s="1">
         <v>45515</v>
       </c>
       <c r="G19" t="s">
@@ -4957,7 +5055,7 @@
       <c r="E20" t="s">
         <v>98</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20" s="1">
         <v>45564</v>
       </c>
       <c r="G20" t="s">
@@ -5010,7 +5108,7 @@
       <c r="E21" t="s">
         <v>98</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21" s="1">
         <v>45564</v>
       </c>
       <c r="G21" t="s">
@@ -5075,7 +5173,7 @@
       <c r="E22" t="s">
         <v>98</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22" s="1">
         <v>45564</v>
       </c>
       <c r="G22" t="s">
@@ -5128,7 +5226,7 @@
       <c r="E23" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23" s="1">
         <v>45564</v>
       </c>
       <c r="G23" t="s">
@@ -5181,7 +5279,7 @@
       <c r="E24" t="s">
         <v>98</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="1">
         <v>45564</v>
       </c>
       <c r="G24" t="s">
@@ -5234,7 +5332,7 @@
       <c r="E25" t="s">
         <v>98</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="1">
         <v>45564</v>
       </c>
       <c r="G25" t="s">
@@ -5287,7 +5385,7 @@
       <c r="E26" t="s">
         <v>98</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="1">
         <v>45564</v>
       </c>
       <c r="G26" t="s">
@@ -5340,7 +5438,7 @@
       <c r="E27" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>45564</v>
       </c>
       <c r="G27" t="s">
@@ -5393,7 +5491,7 @@
       <c r="E28" t="s">
         <v>98</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="1">
         <v>45564</v>
       </c>
       <c r="G28" t="s">
@@ -5446,7 +5544,7 @@
       <c r="E29" t="s">
         <v>98</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="1">
         <v>45564</v>
       </c>
       <c r="G29" t="s">
@@ -5499,7 +5597,7 @@
       <c r="E30" t="s">
         <v>98</v>
       </c>
-      <c r="F30" s="2">
+      <c r="F30" s="1">
         <v>45564</v>
       </c>
       <c r="G30" t="s">
@@ -5552,7 +5650,7 @@
       <c r="E31" t="s">
         <v>98</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="1">
         <v>45564</v>
       </c>
       <c r="G31" t="s">
@@ -5605,7 +5703,7 @@
       <c r="E32" t="s">
         <v>98</v>
       </c>
-      <c r="F32" s="2">
+      <c r="F32" s="1">
         <v>45564</v>
       </c>
       <c r="G32" t="s">
@@ -5658,7 +5756,7 @@
       <c r="E33" t="s">
         <v>98</v>
       </c>
-      <c r="F33" s="2">
+      <c r="F33" s="1">
         <v>45564</v>
       </c>
       <c r="G33" t="s">
@@ -5711,7 +5809,7 @@
       <c r="E34" t="s">
         <v>98</v>
       </c>
-      <c r="F34" s="2">
+      <c r="F34" s="1">
         <v>45564</v>
       </c>
       <c r="G34" t="s">
@@ -5764,7 +5862,7 @@
       <c r="E35" t="s">
         <v>98</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F35" s="1">
         <v>45564</v>
       </c>
       <c r="G35" t="s">
@@ -5817,7 +5915,7 @@
       <c r="E36" t="s">
         <v>98</v>
       </c>
-      <c r="F36" s="2">
+      <c r="F36" s="1">
         <v>45564</v>
       </c>
       <c r="G36" t="s">
@@ -5870,7 +5968,7 @@
       <c r="E37" t="s">
         <v>98</v>
       </c>
-      <c r="F37" s="2">
+      <c r="F37" s="1">
         <v>45564</v>
       </c>
       <c r="G37" t="s">
@@ -5923,7 +6021,7 @@
       <c r="E38" t="s">
         <v>98</v>
       </c>
-      <c r="F38" s="2">
+      <c r="F38" s="1">
         <v>45564</v>
       </c>
       <c r="G38" t="s">
@@ -5976,7 +6074,7 @@
       <c r="E39" t="s">
         <v>98</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F39" s="1">
         <v>45564</v>
       </c>
       <c r="G39" t="s">
@@ -6029,7 +6127,7 @@
       <c r="E40" t="s">
         <v>98</v>
       </c>
-      <c r="F40" s="2">
+      <c r="F40" s="1">
         <v>45564</v>
       </c>
       <c r="G40" t="s">
@@ -6082,7 +6180,7 @@
       <c r="E41" t="s">
         <v>98</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F41" s="1">
         <v>45564</v>
       </c>
       <c r="G41" t="s">
@@ -6135,7 +6233,7 @@
       <c r="E42" t="s">
         <v>98</v>
       </c>
-      <c r="F42" s="2">
+      <c r="F42" s="1">
         <v>45564</v>
       </c>
       <c r="G42" t="s">
@@ -6188,7 +6286,7 @@
       <c r="E43" t="s">
         <v>98</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>45564</v>
       </c>
       <c r="G43" t="s">
@@ -6241,7 +6339,7 @@
       <c r="E44" t="s">
         <v>98</v>
       </c>
-      <c r="F44" s="2">
+      <c r="F44" s="1">
         <v>45564</v>
       </c>
       <c r="G44" t="s">
@@ -6294,7 +6392,7 @@
       <c r="E45" t="s">
         <v>98</v>
       </c>
-      <c r="F45" s="2">
+      <c r="F45" s="1">
         <v>45564</v>
       </c>
       <c r="G45" t="s">
@@ -6347,7 +6445,7 @@
       <c r="E46" t="s">
         <v>98</v>
       </c>
-      <c r="F46" s="2">
+      <c r="F46" s="1">
         <v>45564</v>
       </c>
       <c r="G46" t="s">
@@ -6400,7 +6498,7 @@
       <c r="E47" t="s">
         <v>200</v>
       </c>
-      <c r="F47" s="2">
+      <c r="F47" s="1">
         <v>45592</v>
       </c>
       <c r="G47" t="s">
@@ -6453,7 +6551,7 @@
       <c r="E48" t="s">
         <v>200</v>
       </c>
-      <c r="F48" s="2">
+      <c r="F48" s="1">
         <v>45592</v>
       </c>
       <c r="G48" t="s">
@@ -6506,7 +6604,7 @@
       <c r="E49" t="s">
         <v>200</v>
       </c>
-      <c r="F49" s="2">
+      <c r="F49" s="1">
         <v>45592</v>
       </c>
       <c r="G49" t="s">
@@ -6559,7 +6657,7 @@
       <c r="E50" t="s">
         <v>200</v>
       </c>
-      <c r="F50" s="2">
+      <c r="F50" s="1">
         <v>45592</v>
       </c>
       <c r="G50" t="s">
@@ -6612,7 +6710,7 @@
       <c r="E51" t="s">
         <v>200</v>
       </c>
-      <c r="F51" s="2">
+      <c r="F51" s="1">
         <v>45592</v>
       </c>
       <c r="G51" t="s">
@@ -6665,7 +6763,7 @@
       <c r="E52" t="s">
         <v>200</v>
       </c>
-      <c r="F52" s="2">
+      <c r="F52" s="1">
         <v>45592</v>
       </c>
       <c r="G52" t="s">
@@ -6718,7 +6816,7 @@
       <c r="E53" t="s">
         <v>200</v>
       </c>
-      <c r="F53" s="2">
+      <c r="F53" s="1">
         <v>45592</v>
       </c>
       <c r="G53" t="s">
@@ -6771,7 +6869,7 @@
       <c r="E54" t="s">
         <v>200</v>
       </c>
-      <c r="F54" s="2">
+      <c r="F54" s="1">
         <v>45592</v>
       </c>
       <c r="G54" t="s">
@@ -6824,7 +6922,7 @@
       <c r="E55" t="s">
         <v>200</v>
       </c>
-      <c r="F55" s="2">
+      <c r="F55" s="1">
         <v>45592</v>
       </c>
       <c r="G55" t="s">
@@ -6877,7 +6975,7 @@
       <c r="E56" t="s">
         <v>200</v>
       </c>
-      <c r="F56" s="2">
+      <c r="F56" s="1">
         <v>45592</v>
       </c>
       <c r="G56" t="s">
@@ -6930,7 +7028,7 @@
       <c r="E57" t="s">
         <v>200</v>
       </c>
-      <c r="F57" s="2">
+      <c r="F57" s="1">
         <v>45592</v>
       </c>
       <c r="G57" t="s">
@@ -6983,7 +7081,7 @@
       <c r="E58" t="s">
         <v>200</v>
       </c>
-      <c r="F58" s="2">
+      <c r="F58" s="1">
         <v>45592</v>
       </c>
       <c r="G58" t="s">
@@ -7036,7 +7134,7 @@
       <c r="E59" t="s">
         <v>200</v>
       </c>
-      <c r="F59" s="2">
+      <c r="F59" s="1">
         <v>45592</v>
       </c>
       <c r="G59" t="s">
@@ -7089,7 +7187,7 @@
       <c r="E60" t="s">
         <v>200</v>
       </c>
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <v>45592</v>
       </c>
       <c r="G60" t="s">
@@ -7142,7 +7240,7 @@
       <c r="E61" t="s">
         <v>200</v>
       </c>
-      <c r="F61" s="2">
+      <c r="F61" s="1">
         <v>45592</v>
       </c>
       <c r="G61" t="s">
@@ -7195,7 +7293,7 @@
       <c r="E62" t="s">
         <v>200</v>
       </c>
-      <c r="F62" s="2">
+      <c r="F62" s="1">
         <v>45592</v>
       </c>
       <c r="G62" t="s">
@@ -7248,7 +7346,7 @@
       <c r="E63" t="s">
         <v>29</v>
       </c>
-      <c r="F63" s="2">
+      <c r="F63" s="1">
         <v>45626</v>
       </c>
       <c r="G63" t="s">
@@ -7301,7 +7399,7 @@
       <c r="E64" t="s">
         <v>29</v>
       </c>
-      <c r="F64" s="2">
+      <c r="F64" s="1">
         <v>45626</v>
       </c>
       <c r="G64" t="s">
@@ -7354,7 +7452,7 @@
       <c r="E65" t="s">
         <v>29</v>
       </c>
-      <c r="F65" s="2">
+      <c r="F65" s="1">
         <v>45626</v>
       </c>
       <c r="G65" t="s">
@@ -7407,7 +7505,7 @@
       <c r="E66" t="s">
         <v>29</v>
       </c>
-      <c r="F66" s="2">
+      <c r="F66" s="1">
         <v>45626</v>
       </c>
       <c r="G66" t="s">
@@ -7460,7 +7558,7 @@
       <c r="E67" t="s">
         <v>29</v>
       </c>
-      <c r="F67" s="2">
+      <c r="F67" s="1">
         <v>45626</v>
       </c>
       <c r="G67" t="s">
@@ -7513,7 +7611,7 @@
       <c r="E68" t="s">
         <v>29</v>
       </c>
-      <c r="F68" s="2">
+      <c r="F68" s="1">
         <v>45626</v>
       </c>
       <c r="G68" t="s">
@@ -7566,7 +7664,7 @@
       <c r="E69" t="s">
         <v>29</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>45626</v>
       </c>
       <c r="G69" t="s">
@@ -7619,7 +7717,7 @@
       <c r="E70" t="s">
         <v>29</v>
       </c>
-      <c r="F70" s="2">
+      <c r="F70" s="1">
         <v>45626</v>
       </c>
       <c r="G70" t="s">
@@ -7672,7 +7770,7 @@
       <c r="E71" t="s">
         <v>29</v>
       </c>
-      <c r="F71" s="2">
+      <c r="F71" s="1">
         <v>45626</v>
       </c>
       <c r="G71" t="s">
@@ -7725,7 +7823,7 @@
       <c r="E72" t="s">
         <v>29</v>
       </c>
-      <c r="F72" s="2">
+      <c r="F72" s="1">
         <v>45626</v>
       </c>
       <c r="G72" t="s">
@@ -7778,7 +7876,7 @@
       <c r="E73" t="s">
         <v>29</v>
       </c>
-      <c r="F73" s="2">
+      <c r="F73" s="1">
         <v>45626</v>
       </c>
       <c r="G73" t="s">
@@ -7831,7 +7929,7 @@
       <c r="E74" t="s">
         <v>29</v>
       </c>
-      <c r="F74" s="2">
+      <c r="F74" s="1">
         <v>45626</v>
       </c>
       <c r="G74" t="s">
@@ -7884,7 +7982,7 @@
       <c r="E75" t="s">
         <v>29</v>
       </c>
-      <c r="F75" s="2">
+      <c r="F75" s="1">
         <v>45626</v>
       </c>
       <c r="G75" t="s">
@@ -7937,7 +8035,7 @@
       <c r="E76" t="s">
         <v>29</v>
       </c>
-      <c r="F76" s="2">
+      <c r="F76" s="1">
         <v>45626</v>
       </c>
       <c r="G76" t="s">
@@ -7990,7 +8088,7 @@
       <c r="E77" t="s">
         <v>29</v>
       </c>
-      <c r="F77" s="2">
+      <c r="F77" s="1">
         <v>45626</v>
       </c>
       <c r="G77" t="s">
@@ -8043,7 +8141,7 @@
       <c r="E78" t="s">
         <v>29</v>
       </c>
-      <c r="F78" s="2">
+      <c r="F78" s="1">
         <v>45626</v>
       </c>
       <c r="G78" t="s">
@@ -8096,7 +8194,7 @@
       <c r="E79" t="s">
         <v>29</v>
       </c>
-      <c r="F79" s="2">
+      <c r="F79" s="1">
         <v>45626</v>
       </c>
       <c r="G79" t="s">
@@ -8149,7 +8247,7 @@
       <c r="E80" t="s">
         <v>29</v>
       </c>
-      <c r="F80" s="2">
+      <c r="F80" s="1">
         <v>45626</v>
       </c>
       <c r="G80" t="s">
@@ -8202,7 +8300,7 @@
       <c r="E81" t="s">
         <v>29</v>
       </c>
-      <c r="F81" s="2">
+      <c r="F81" s="1">
         <v>45626</v>
       </c>
       <c r="G81" t="s">
@@ -8255,7 +8353,7 @@
       <c r="E82" t="s">
         <v>29</v>
       </c>
-      <c r="F82" s="2">
+      <c r="F82" s="1">
         <v>45626</v>
       </c>
       <c r="G82" t="s">
@@ -8308,7 +8406,7 @@
       <c r="E83" t="s">
         <v>29</v>
       </c>
-      <c r="F83" s="2">
+      <c r="F83" s="1">
         <v>45626</v>
       </c>
       <c r="G83" t="s">
@@ -8361,7 +8459,7 @@
       <c r="E84" t="s">
         <v>29</v>
       </c>
-      <c r="F84" s="2">
+      <c r="F84" s="1">
         <v>45626</v>
       </c>
       <c r="G84" t="s">
@@ -8414,7 +8512,7 @@
       <c r="E85" t="s">
         <v>29</v>
       </c>
-      <c r="F85" s="2">
+      <c r="F85" s="1">
         <v>45626</v>
       </c>
       <c r="G85" t="s">
@@ -8467,7 +8565,7 @@
       <c r="E86" t="s">
         <v>29</v>
       </c>
-      <c r="F86" s="2">
+      <c r="F86" s="1">
         <v>45807</v>
       </c>
       <c r="G86" t="s">
@@ -8532,7 +8630,7 @@
       <c r="E87" t="s">
         <v>29</v>
       </c>
-      <c r="F87" s="2">
+      <c r="F87" s="1">
         <v>45807</v>
       </c>
       <c r="G87" t="s">
@@ -8597,7 +8695,7 @@
       <c r="E88" t="s">
         <v>29</v>
       </c>
-      <c r="F88" s="2">
+      <c r="F88" s="1">
         <v>45807</v>
       </c>
       <c r="G88" t="s">
@@ -8671,7 +8769,7 @@
       <c r="E89" t="s">
         <v>29</v>
       </c>
-      <c r="F89" s="2">
+      <c r="F89" s="1">
         <v>45807</v>
       </c>
       <c r="G89" t="s">
@@ -8736,7 +8834,7 @@
       <c r="E90" t="s">
         <v>29</v>
       </c>
-      <c r="F90" s="2">
+      <c r="F90" s="1">
         <v>45807</v>
       </c>
       <c r="G90" t="s">
@@ -8810,7 +8908,7 @@
       <c r="E91" t="s">
         <v>29</v>
       </c>
-      <c r="F91" s="2">
+      <c r="F91" s="1">
         <v>45808</v>
       </c>
       <c r="G91" t="s">
@@ -8884,7 +8982,7 @@
       <c r="E92" t="s">
         <v>29</v>
       </c>
-      <c r="F92" s="2">
+      <c r="F92" s="1">
         <v>45808</v>
       </c>
       <c r="G92" t="s">
@@ -8958,7 +9056,7 @@
       <c r="E93" t="s">
         <v>29</v>
       </c>
-      <c r="F93" s="2">
+      <c r="F93" s="1">
         <v>45808</v>
       </c>
       <c r="G93" t="s">
@@ -9023,7 +9121,7 @@
       <c r="E94" t="s">
         <v>29</v>
       </c>
-      <c r="F94" s="2">
+      <c r="F94" s="1">
         <v>45808</v>
       </c>
       <c r="G94" t="s">
@@ -9097,7 +9195,7 @@
       <c r="E95" t="s">
         <v>29</v>
       </c>
-      <c r="F95" s="2">
+      <c r="F95" s="1">
         <v>45808</v>
       </c>
       <c r="G95" t="s">
@@ -9171,7 +9269,7 @@
       <c r="E96" t="s">
         <v>29</v>
       </c>
-      <c r="F96" s="2">
+      <c r="F96" s="1">
         <v>45808</v>
       </c>
       <c r="G96" t="s">
@@ -9245,7 +9343,7 @@
       <c r="E97" t="s">
         <v>29</v>
       </c>
-      <c r="F97" s="2">
+      <c r="F97" s="1">
         <v>45808</v>
       </c>
       <c r="G97" t="s">
@@ -9310,7 +9408,7 @@
       <c r="E98" t="s">
         <v>29</v>
       </c>
-      <c r="F98" s="2">
+      <c r="F98" s="1">
         <v>45808</v>
       </c>
       <c r="G98" t="s">
@@ -9384,7 +9482,7 @@
       <c r="E99" t="s">
         <v>29</v>
       </c>
-      <c r="F99" s="2">
+      <c r="F99" s="1">
         <v>45808</v>
       </c>
       <c r="G99" t="s">
@@ -9458,7 +9556,7 @@
       <c r="E100" t="s">
         <v>29</v>
       </c>
-      <c r="F100" s="2">
+      <c r="F100" s="1">
         <v>45808</v>
       </c>
       <c r="G100" t="s">
@@ -9523,7 +9621,7 @@
       <c r="E101" t="s">
         <v>29</v>
       </c>
-      <c r="F101" s="2">
+      <c r="F101" s="1">
         <v>45808</v>
       </c>
       <c r="G101" t="s">
@@ -9597,7 +9695,7 @@
       <c r="E102" t="s">
         <v>403</v>
       </c>
-      <c r="F102" s="2">
+      <c r="F102" s="1">
         <v>45844</v>
       </c>
       <c r="G102" t="s">
@@ -9650,7 +9748,7 @@
       <c r="E103" t="s">
         <v>403</v>
       </c>
-      <c r="F103" s="2">
+      <c r="F103" s="1">
         <v>45844</v>
       </c>
       <c r="G103" t="s">
@@ -9703,7 +9801,7 @@
       <c r="E104" t="s">
         <v>403</v>
       </c>
-      <c r="F104" s="2">
+      <c r="F104" s="1">
         <v>45844</v>
       </c>
       <c r="G104" t="s">
@@ -9753,7 +9851,7 @@
       <c r="E105" t="s">
         <v>403</v>
       </c>
-      <c r="F105" s="2">
+      <c r="F105" s="1">
         <v>45844</v>
       </c>
       <c r="G105" t="s">
@@ -9803,7 +9901,7 @@
       <c r="E106" t="s">
         <v>403</v>
       </c>
-      <c r="F106" s="2">
+      <c r="F106" s="1">
         <v>45844</v>
       </c>
       <c r="G106" t="s">
@@ -9853,7 +9951,7 @@
       <c r="E107" t="s">
         <v>403</v>
       </c>
-      <c r="F107" s="2">
+      <c r="F107" s="1">
         <v>45844</v>
       </c>
       <c r="G107" t="s">
@@ -9903,7 +10001,7 @@
       <c r="E108" t="s">
         <v>403</v>
       </c>
-      <c r="F108" s="2">
+      <c r="F108" s="1">
         <v>45844</v>
       </c>
       <c r="G108" t="s">
@@ -9953,7 +10051,7 @@
       <c r="E109" t="s">
         <v>403</v>
       </c>
-      <c r="F109" s="2">
+      <c r="F109" s="1">
         <v>45844</v>
       </c>
       <c r="G109" t="s">
@@ -10003,7 +10101,7 @@
       <c r="E110" t="s">
         <v>403</v>
       </c>
-      <c r="F110" s="2">
+      <c r="F110" s="1">
         <v>45844</v>
       </c>
       <c r="G110" t="s">
@@ -10056,7 +10154,7 @@
       <c r="E111" t="s">
         <v>200</v>
       </c>
-      <c r="F111" s="2">
+      <c r="F111" s="1">
         <v>45858</v>
       </c>
       <c r="G111" t="s">
@@ -10130,7 +10228,7 @@
       <c r="E112" t="s">
         <v>200</v>
       </c>
-      <c r="F112" s="2">
+      <c r="F112" s="1">
         <v>45858</v>
       </c>
       <c r="G112" t="s">
@@ -10204,7 +10302,7 @@
       <c r="E113" t="s">
         <v>200</v>
       </c>
-      <c r="F113" s="2">
+      <c r="F113" s="1">
         <v>45858</v>
       </c>
       <c r="G113" t="s">
@@ -10278,7 +10376,7 @@
       <c r="E114" t="s">
         <v>200</v>
       </c>
-      <c r="F114" s="2">
+      <c r="F114" s="1">
         <v>45858</v>
       </c>
       <c r="G114" t="s">
@@ -10352,7 +10450,7 @@
       <c r="E115" t="s">
         <v>200</v>
       </c>
-      <c r="F115" s="2">
+      <c r="F115" s="1">
         <v>45858</v>
       </c>
       <c r="G115" t="s">
@@ -10426,7 +10524,7 @@
       <c r="E116" t="s">
         <v>200</v>
       </c>
-      <c r="F116" s="2">
+      <c r="F116" s="1">
         <v>45858</v>
       </c>
       <c r="G116" t="s">
@@ -10491,7 +10589,7 @@
       <c r="E117" t="s">
         <v>200</v>
       </c>
-      <c r="F117" s="2">
+      <c r="F117" s="1">
         <v>45858</v>
       </c>
       <c r="G117" t="s">
@@ -10556,7 +10654,7 @@
       <c r="E118" t="s">
         <v>200</v>
       </c>
-      <c r="F118" s="2">
+      <c r="F118" s="1">
         <v>45858</v>
       </c>
       <c r="G118" t="s">
@@ -10630,7 +10728,7 @@
       <c r="E119" t="s">
         <v>200</v>
       </c>
-      <c r="F119" s="2">
+      <c r="F119" s="1">
         <v>45858</v>
       </c>
       <c r="G119" t="s">
@@ -10704,7 +10802,7 @@
       <c r="E120" t="s">
         <v>200</v>
       </c>
-      <c r="F120" s="2">
+      <c r="F120" s="1">
         <v>45858</v>
       </c>
       <c r="G120" t="s">
@@ -10778,7 +10876,7 @@
       <c r="E121" t="s">
         <v>200</v>
       </c>
-      <c r="F121" s="2">
+      <c r="F121" s="1">
         <v>45858</v>
       </c>
       <c r="G121" t="s">
@@ -10849,7 +10947,7 @@
       <c r="E122" t="s">
         <v>403</v>
       </c>
-      <c r="F122" s="2">
+      <c r="F122" s="1">
         <v>45879</v>
       </c>
       <c r="G122" t="s">
@@ -10899,7 +10997,7 @@
       <c r="E123" t="s">
         <v>403</v>
       </c>
-      <c r="F123" s="2">
+      <c r="F123" s="1">
         <v>45879</v>
       </c>
       <c r="G123" t="s">
@@ -10949,7 +11047,7 @@
       <c r="E124" t="s">
         <v>403</v>
       </c>
-      <c r="F124" s="2">
+      <c r="F124" s="1">
         <v>45879</v>
       </c>
       <c r="G124" t="s">
@@ -10999,7 +11097,7 @@
       <c r="E125" t="s">
         <v>403</v>
       </c>
-      <c r="F125" s="2">
+      <c r="F125" s="1">
         <v>45879</v>
       </c>
       <c r="G125" t="s">
@@ -11049,7 +11147,7 @@
       <c r="E126" t="s">
         <v>403</v>
       </c>
-      <c r="F126" s="2">
+      <c r="F126" s="1">
         <v>45879</v>
       </c>
       <c r="G126" t="s">
@@ -11099,7 +11197,7 @@
       <c r="E127" t="s">
         <v>403</v>
       </c>
-      <c r="F127" s="2">
+      <c r="F127" s="1">
         <v>45879</v>
       </c>
       <c r="G127" t="s">
@@ -11149,7 +11247,7 @@
       <c r="E128" t="s">
         <v>403</v>
       </c>
-      <c r="F128" s="2">
+      <c r="F128" s="1">
         <v>45879</v>
       </c>
       <c r="G128" t="s">
@@ -11199,7 +11297,7 @@
       <c r="E129" t="s">
         <v>403</v>
       </c>
-      <c r="F129" s="2">
+      <c r="F129" s="1">
         <v>45879</v>
       </c>
       <c r="G129" t="s">
@@ -11249,7 +11347,7 @@
       <c r="E130" t="s">
         <v>403</v>
       </c>
-      <c r="F130" s="2">
+      <c r="F130" s="1">
         <v>45879</v>
       </c>
       <c r="G130" t="s">
@@ -11299,7 +11397,7 @@
       <c r="E131" t="s">
         <v>403</v>
       </c>
-      <c r="F131" s="2">
+      <c r="F131" s="1">
         <v>45914</v>
       </c>
       <c r="G131" t="s">
@@ -11349,7 +11447,7 @@
       <c r="E132" t="s">
         <v>403</v>
       </c>
-      <c r="F132" s="2">
+      <c r="F132" s="1">
         <v>45914</v>
       </c>
       <c r="G132" t="s">
@@ -11399,7 +11497,7 @@
       <c r="E133" t="s">
         <v>403</v>
       </c>
-      <c r="F133" s="2">
+      <c r="F133" s="1">
         <v>45914</v>
       </c>
       <c r="G133" t="s">
@@ -11449,7 +11547,7 @@
       <c r="E134" t="s">
         <v>403</v>
       </c>
-      <c r="F134" s="2">
+      <c r="F134" s="1">
         <v>45914</v>
       </c>
       <c r="G134" t="s">
@@ -11499,7 +11597,7 @@
       <c r="E135" t="s">
         <v>403</v>
       </c>
-      <c r="F135" s="2">
+      <c r="F135" s="1">
         <v>45914</v>
       </c>
       <c r="G135" t="s">
@@ -11549,7 +11647,7 @@
       <c r="E136" t="s">
         <v>403</v>
       </c>
-      <c r="F136" s="2">
+      <c r="F136" s="1">
         <v>45914</v>
       </c>
       <c r="G136" t="s">
@@ -11599,7 +11697,7 @@
       <c r="E137" t="s">
         <v>403</v>
       </c>
-      <c r="F137" s="2">
+      <c r="F137" s="1">
         <v>45914</v>
       </c>
       <c r="G137" t="s">
@@ -11649,7 +11747,7 @@
       <c r="E138" t="s">
         <v>403</v>
       </c>
-      <c r="F138" s="2">
+      <c r="F138" s="1">
         <v>45914</v>
       </c>
       <c r="G138" t="s">
@@ -11699,7 +11797,7 @@
       <c r="E139" t="s">
         <v>403</v>
       </c>
-      <c r="F139" s="2">
+      <c r="F139" s="1">
         <v>45914</v>
       </c>
       <c r="G139" t="s">
@@ -11749,7 +11847,7 @@
       <c r="E140" t="s">
         <v>403</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140" s="1">
         <v>45914</v>
       </c>
       <c r="G140" t="s">
@@ -11799,7 +11897,7 @@
       <c r="E141" t="s">
         <v>403</v>
       </c>
-      <c r="F141" s="2">
+      <c r="F141" s="1">
         <v>45914</v>
       </c>
       <c r="G141" t="s">
@@ -11849,7 +11947,7 @@
       <c r="E142" t="s">
         <v>403</v>
       </c>
-      <c r="F142" s="2">
+      <c r="F142" s="1">
         <v>45914</v>
       </c>
       <c r="G142" t="s">
@@ -11899,7 +11997,7 @@
       <c r="E143" t="s">
         <v>403</v>
       </c>
-      <c r="F143" s="2">
+      <c r="F143" s="1">
         <v>45914</v>
       </c>
       <c r="G143" t="s">
@@ -11949,7 +12047,7 @@
       <c r="E144" t="s">
         <v>403</v>
       </c>
-      <c r="F144" s="2">
+      <c r="F144" s="1">
         <v>45914</v>
       </c>
       <c r="G144" t="s">
@@ -11999,7 +12097,7 @@
       <c r="E145" t="s">
         <v>403</v>
       </c>
-      <c r="F145" s="2">
+      <c r="F145" s="1">
         <v>45914</v>
       </c>
       <c r="G145" t="s">
@@ -12049,7 +12147,7 @@
       <c r="E146" t="s">
         <v>403</v>
       </c>
-      <c r="F146" s="2">
+      <c r="F146" s="1">
         <v>45914</v>
       </c>
       <c r="G146" t="s">
@@ -12099,7 +12197,7 @@
       <c r="E147" t="s">
         <v>403</v>
       </c>
-      <c r="F147" s="2">
+      <c r="F147" s="1">
         <v>45914</v>
       </c>
       <c r="G147" t="s">
@@ -12149,7 +12247,7 @@
       <c r="E148" t="s">
         <v>403</v>
       </c>
-      <c r="F148" s="2">
+      <c r="F148" s="1">
         <v>45914</v>
       </c>
       <c r="G148" t="s">
@@ -12202,7 +12300,7 @@
       <c r="E149" t="s">
         <v>29</v>
       </c>
-      <c r="F149" s="2">
+      <c r="F149" s="1">
         <v>45920</v>
       </c>
       <c r="G149" t="s">
@@ -12255,7 +12353,7 @@
       <c r="E150" t="s">
         <v>29</v>
       </c>
-      <c r="F150" s="2">
+      <c r="F150" s="1">
         <v>45920</v>
       </c>
       <c r="G150" t="s">
@@ -12308,7 +12406,7 @@
       <c r="E151" t="s">
         <v>29</v>
       </c>
-      <c r="F151" s="2">
+      <c r="F151" s="1">
         <v>45920</v>
       </c>
       <c r="G151" t="s">
@@ -12373,7 +12471,7 @@
       <c r="E152" t="s">
         <v>29</v>
       </c>
-      <c r="F152" s="2">
+      <c r="F152" s="1">
         <v>45920</v>
       </c>
       <c r="G152" t="s">
@@ -12438,7 +12536,7 @@
       <c r="E153" t="s">
         <v>29</v>
       </c>
-      <c r="F153" s="2">
+      <c r="F153" s="1">
         <v>45920</v>
       </c>
       <c r="G153" t="s">
@@ -12512,7 +12610,7 @@
       <c r="E154" t="s">
         <v>29</v>
       </c>
-      <c r="F154" s="2">
+      <c r="F154" s="1">
         <v>45920</v>
       </c>
       <c r="G154" t="s">
@@ -12574,7 +12672,7 @@
       <c r="E155" t="s">
         <v>29</v>
       </c>
-      <c r="F155" s="2">
+      <c r="F155" s="1">
         <v>45920</v>
       </c>
       <c r="G155" t="s">
@@ -12636,7 +12734,7 @@
       <c r="E156" t="s">
         <v>29</v>
       </c>
-      <c r="F156" s="2">
+      <c r="F156" s="1">
         <v>45920</v>
       </c>
       <c r="G156" t="s">
@@ -12698,7 +12796,7 @@
       <c r="E157" t="s">
         <v>29</v>
       </c>
-      <c r="F157" s="2">
+      <c r="F157" s="1">
         <v>45920</v>
       </c>
       <c r="G157" t="s">
@@ -12769,7 +12867,7 @@
       <c r="E158" t="s">
         <v>29</v>
       </c>
-      <c r="F158" s="2">
+      <c r="F158" s="1">
         <v>45920</v>
       </c>
       <c r="G158" t="s">
@@ -12822,7 +12920,7 @@
       <c r="E159" t="s">
         <v>403</v>
       </c>
-      <c r="F159" s="2">
+      <c r="F159" s="1">
         <v>45935</v>
       </c>
       <c r="G159" t="s">
@@ -12887,7 +12985,7 @@
       <c r="E160" t="s">
         <v>403</v>
       </c>
-      <c r="F160" s="2">
+      <c r="F160" s="1">
         <v>45935</v>
       </c>
       <c r="G160" t="s">
@@ -12961,7 +13059,7 @@
       <c r="E161" t="s">
         <v>403</v>
       </c>
-      <c r="F161" s="2">
+      <c r="F161" s="1">
         <v>45935</v>
       </c>
       <c r="G161" t="s">
@@ -13035,7 +13133,7 @@
       <c r="E162" t="s">
         <v>403</v>
       </c>
-      <c r="F162" s="2">
+      <c r="F162" s="1">
         <v>45935</v>
       </c>
       <c r="G162" t="s">
@@ -13109,7 +13207,7 @@
       <c r="E163" t="s">
         <v>403</v>
       </c>
-      <c r="F163" s="2">
+      <c r="F163" s="1">
         <v>45935</v>
       </c>
       <c r="G163" t="s">
@@ -13183,7 +13281,7 @@
       <c r="E164" t="s">
         <v>403</v>
       </c>
-      <c r="F164" s="2">
+      <c r="F164" s="1">
         <v>45935</v>
       </c>
       <c r="G164" t="s">
@@ -13257,7 +13355,7 @@
       <c r="E165" t="s">
         <v>403</v>
       </c>
-      <c r="F165" s="2">
+      <c r="F165" s="1">
         <v>45935</v>
       </c>
       <c r="G165" t="s">
@@ -13331,7 +13429,7 @@
       <c r="E166" t="s">
         <v>403</v>
       </c>
-      <c r="F166" s="2">
+      <c r="F166" s="1">
         <v>45935</v>
       </c>
       <c r="G166" t="s">
@@ -13405,7 +13503,7 @@
       <c r="E167" t="s">
         <v>403</v>
       </c>
-      <c r="F167" s="2">
+      <c r="F167" s="1">
         <v>45935</v>
       </c>
       <c r="G167" t="s">
@@ -13479,7 +13577,7 @@
       <c r="E168" t="s">
         <v>403</v>
       </c>
-      <c r="F168" s="2">
+      <c r="F168" s="1">
         <v>45935</v>
       </c>
       <c r="G168" t="s">
@@ -13553,7 +13651,7 @@
       <c r="E169" t="s">
         <v>29</v>
       </c>
-      <c r="F169" s="2">
+      <c r="F169" s="1">
         <v>45951</v>
       </c>
       <c r="G169" t="s">
@@ -13618,7 +13716,7 @@
       <c r="E170" t="s">
         <v>29</v>
       </c>
-      <c r="F170" s="2">
+      <c r="F170" s="1">
         <v>45951</v>
       </c>
       <c r="G170" t="s">
@@ -13683,7 +13781,7 @@
       <c r="E171" t="s">
         <v>29</v>
       </c>
-      <c r="F171" s="2">
+      <c r="F171" s="1">
         <v>45951</v>
       </c>
       <c r="G171" t="s">
@@ -13757,11 +13855,11 @@
       <c r="E172" t="s">
         <v>29</v>
       </c>
-      <c r="F172" s="2">
+      <c r="F172" s="1">
         <v>45951</v>
       </c>
       <c r="G172" t="s">
-        <v>418</v>
+        <v>625</v>
       </c>
       <c r="H172">
         <v>1</v>
@@ -13776,7 +13874,7 @@
         <v>346</v>
       </c>
       <c r="L172" t="s">
-        <v>418</v>
+        <v>625</v>
       </c>
       <c r="M172" t="s">
         <v>29</v>
@@ -13822,7 +13920,7 @@
       <c r="E173" t="s">
         <v>29</v>
       </c>
-      <c r="F173" s="2">
+      <c r="F173" s="1">
         <v>45951</v>
       </c>
       <c r="G173" t="s">
@@ -13896,7 +13994,7 @@
       <c r="E174" t="s">
         <v>29</v>
       </c>
-      <c r="F174" s="2">
+      <c r="F174" s="1">
         <v>45951</v>
       </c>
       <c r="G174" t="s">
@@ -13970,7 +14068,7 @@
       <c r="E175" t="s">
         <v>29</v>
       </c>
-      <c r="F175" s="2">
+      <c r="F175" s="1">
         <v>45951</v>
       </c>
       <c r="G175" t="s">
@@ -14047,7 +14145,7 @@
       <c r="E176" t="s">
         <v>29</v>
       </c>
-      <c r="F176" s="2">
+      <c r="F176" s="1">
         <v>45951</v>
       </c>
       <c r="G176" t="s">
@@ -14118,7 +14216,7 @@
       <c r="E177" t="s">
         <v>403</v>
       </c>
-      <c r="F177" s="2">
+      <c r="F177" s="1">
         <v>45956</v>
       </c>
       <c r="G177" t="s">
@@ -14168,7 +14266,7 @@
       <c r="E178" t="s">
         <v>403</v>
       </c>
-      <c r="F178" s="2">
+      <c r="F178" s="1">
         <v>45956</v>
       </c>
       <c r="G178" t="s">
@@ -14218,7 +14316,7 @@
       <c r="E179" t="s">
         <v>403</v>
       </c>
-      <c r="F179" s="2">
+      <c r="F179" s="1">
         <v>45956</v>
       </c>
       <c r="G179" t="s">
@@ -14268,7 +14366,7 @@
       <c r="E180" t="s">
         <v>403</v>
       </c>
-      <c r="F180" s="2">
+      <c r="F180" s="1">
         <v>45956</v>
       </c>
       <c r="G180" t="s">
@@ -14318,7 +14416,7 @@
       <c r="E181" t="s">
         <v>403</v>
       </c>
-      <c r="F181" s="2">
+      <c r="F181" s="1">
         <v>45956</v>
       </c>
       <c r="G181" t="s">
@@ -14368,7 +14466,7 @@
       <c r="E182" t="s">
         <v>403</v>
       </c>
-      <c r="F182" s="2">
+      <c r="F182" s="1">
         <v>45956</v>
       </c>
       <c r="G182" t="s">
@@ -14418,7 +14516,7 @@
       <c r="E183" t="s">
         <v>403</v>
       </c>
-      <c r="F183" s="2">
+      <c r="F183" s="1">
         <v>45956</v>
       </c>
       <c r="G183" t="s">
@@ -14468,7 +14566,7 @@
       <c r="E184" t="s">
         <v>403</v>
       </c>
-      <c r="F184" s="2">
+      <c r="F184" s="1">
         <v>45956</v>
       </c>
       <c r="G184" t="s">
@@ -14518,7 +14616,7 @@
       <c r="E185" t="s">
         <v>403</v>
       </c>
-      <c r="F185" s="2">
+      <c r="F185" s="1">
         <v>45956</v>
       </c>
       <c r="G185" t="s">
@@ -14568,7 +14666,7 @@
       <c r="E186" t="s">
         <v>403</v>
       </c>
-      <c r="F186" s="2">
+      <c r="F186" s="1">
         <v>45956</v>
       </c>
       <c r="G186" t="s">
@@ -14618,7 +14716,7 @@
       <c r="E187" t="s">
         <v>403</v>
       </c>
-      <c r="F187" s="2">
+      <c r="F187" s="1">
         <v>45956</v>
       </c>
       <c r="G187" t="s">
@@ -14668,7 +14766,7 @@
       <c r="E188" t="s">
         <v>403</v>
       </c>
-      <c r="F188" s="2">
+      <c r="F188" s="1">
         <v>45956</v>
       </c>
       <c r="G188" t="s">
@@ -14721,7 +14819,7 @@
       <c r="E189" t="s">
         <v>403</v>
       </c>
-      <c r="F189" s="2">
+      <c r="F189" s="1">
         <v>45956</v>
       </c>
       <c r="G189" t="s">
@@ -14786,7 +14884,7 @@
       <c r="E190" t="s">
         <v>403</v>
       </c>
-      <c r="F190" s="2">
+      <c r="F190" s="1">
         <v>45956</v>
       </c>
       <c r="G190" t="s">
@@ -14857,7 +14955,7 @@
       <c r="E191" t="s">
         <v>403</v>
       </c>
-      <c r="F191" s="2">
+      <c r="F191" s="1">
         <v>45956</v>
       </c>
       <c r="G191" t="s">
@@ -14907,7 +15005,7 @@
       <c r="E192" t="s">
         <v>403</v>
       </c>
-      <c r="F192" s="2">
+      <c r="F192" s="1">
         <v>45956</v>
       </c>
       <c r="G192" t="s">
@@ -14969,7 +15067,7 @@
       <c r="E193" t="s">
         <v>403</v>
       </c>
-      <c r="F193" s="2">
+      <c r="F193" s="1">
         <v>45956</v>
       </c>
       <c r="G193" t="s">
@@ -15022,7 +15120,7 @@
       <c r="E194" t="s">
         <v>403</v>
       </c>
-      <c r="F194" s="2">
+      <c r="F194" s="1">
         <v>45956</v>
       </c>
       <c r="G194" t="s">
@@ -15087,7 +15185,7 @@
       <c r="E195" t="s">
         <v>403</v>
       </c>
-      <c r="F195" s="2">
+      <c r="F195" s="1">
         <v>45956</v>
       </c>
       <c r="G195" t="s">
@@ -15158,7 +15256,7 @@
       <c r="E196" t="s">
         <v>403</v>
       </c>
-      <c r="F196" s="2">
+      <c r="F196" s="1">
         <v>45956</v>
       </c>
       <c r="G196" t="s">
@@ -15208,7 +15306,7 @@
       <c r="E197" t="s">
         <v>403</v>
       </c>
-      <c r="F197" s="2">
+      <c r="F197" s="1">
         <v>45956</v>
       </c>
       <c r="G197" t="s">
@@ -15258,7 +15356,7 @@
       <c r="E198" t="s">
         <v>403</v>
       </c>
-      <c r="F198" s="2">
+      <c r="F198" s="1">
         <v>45956</v>
       </c>
       <c r="G198" t="s">
@@ -15308,7 +15406,7 @@
       <c r="E199" t="s">
         <v>403</v>
       </c>
-      <c r="F199" s="2">
+      <c r="F199" s="1">
         <v>45956</v>
       </c>
       <c r="G199" t="s">
@@ -15361,7 +15459,7 @@
       <c r="E200" t="s">
         <v>29</v>
       </c>
-      <c r="F200" s="2">
+      <c r="F200" s="1">
         <v>45962</v>
       </c>
       <c r="G200" t="s">
@@ -15414,7 +15512,7 @@
       <c r="E201" t="s">
         <v>29</v>
       </c>
-      <c r="F201" s="2">
+      <c r="F201" s="1">
         <v>45962</v>
       </c>
       <c r="G201" t="s">
@@ -15467,7 +15565,7 @@
       <c r="E202" t="s">
         <v>29</v>
       </c>
-      <c r="F202" s="2">
+      <c r="F202" s="1">
         <v>45962</v>
       </c>
       <c r="G202" t="s">
@@ -15520,7 +15618,7 @@
       <c r="E203" t="s">
         <v>29</v>
       </c>
-      <c r="F203" s="2">
+      <c r="F203" s="1">
         <v>45962</v>
       </c>
       <c r="G203" t="s">
@@ -15585,7 +15683,7 @@
       <c r="E204" t="s">
         <v>29</v>
       </c>
-      <c r="F204" s="2">
+      <c r="F204" s="1">
         <v>45962</v>
       </c>
       <c r="G204" t="s">
@@ -15659,7 +15757,7 @@
       <c r="E205" t="s">
         <v>29</v>
       </c>
-      <c r="F205" s="2">
+      <c r="F205" s="1">
         <v>45962</v>
       </c>
       <c r="G205" t="s">
@@ -15733,7 +15831,7 @@
       <c r="E206" t="s">
         <v>29</v>
       </c>
-      <c r="F206" s="2">
+      <c r="F206" s="1">
         <v>45962</v>
       </c>
       <c r="G206" t="s">
@@ -15786,7 +15884,7 @@
       <c r="E207" t="s">
         <v>29</v>
       </c>
-      <c r="F207" s="2">
+      <c r="F207" s="1">
         <v>45963</v>
       </c>
       <c r="G207" t="s">
@@ -15860,7 +15958,7 @@
       <c r="E208" t="s">
         <v>29</v>
       </c>
-      <c r="F208" s="2">
+      <c r="F208" s="1">
         <v>45963</v>
       </c>
       <c r="G208" t="s">
@@ -15937,7 +16035,7 @@
       <c r="E209" t="s">
         <v>29</v>
       </c>
-      <c r="F209" s="2">
+      <c r="F209" s="1">
         <v>45963</v>
       </c>
       <c r="G209" t="s">
@@ -16014,7 +16112,7 @@
       <c r="E210" t="s">
         <v>29</v>
       </c>
-      <c r="F210" s="2">
+      <c r="F210" s="1">
         <v>45963</v>
       </c>
       <c r="G210" t="s">
@@ -16091,7 +16189,7 @@
       <c r="E211" t="s">
         <v>29</v>
       </c>
-      <c r="F211" s="2">
+      <c r="F211" s="1">
         <v>45963</v>
       </c>
       <c r="G211" t="s">
@@ -16168,7 +16266,7 @@
       <c r="E212" t="s">
         <v>29</v>
       </c>
-      <c r="F212" s="2">
+      <c r="F212" s="1">
         <v>45963</v>
       </c>
       <c r="G212" t="s">
@@ -16245,7 +16343,7 @@
       <c r="E213" t="s">
         <v>29</v>
       </c>
-      <c r="F213" s="2">
+      <c r="F213" s="1">
         <v>45963</v>
       </c>
       <c r="G213" t="s">
@@ -16322,7 +16420,7 @@
       <c r="E214" t="s">
         <v>29</v>
       </c>
-      <c r="F214" s="2">
+      <c r="F214" s="1">
         <v>45963</v>
       </c>
       <c r="G214" t="s">
@@ -16399,7 +16497,7 @@
       <c r="E215" t="s">
         <v>29</v>
       </c>
-      <c r="F215" s="2">
+      <c r="F215" s="1">
         <v>45963</v>
       </c>
       <c r="G215" t="s">
@@ -16476,7 +16574,7 @@
       <c r="E216" t="s">
         <v>29</v>
       </c>
-      <c r="F216" s="2">
+      <c r="F216" s="1">
         <v>45963</v>
       </c>
       <c r="G216" t="s">
@@ -16553,7 +16651,7 @@
       <c r="E217" t="s">
         <v>29</v>
       </c>
-      <c r="F217" s="2">
+      <c r="F217" s="1">
         <v>45963</v>
       </c>
       <c r="G217" t="s">
@@ -16627,7 +16725,7 @@
       <c r="E218" t="s">
         <v>29</v>
       </c>
-      <c r="F218" s="2">
+      <c r="F218" s="1">
         <v>45963</v>
       </c>
       <c r="G218" t="s">
@@ -16701,7 +16799,7 @@
       <c r="E219" t="s">
         <v>29</v>
       </c>
-      <c r="F219" s="2">
+      <c r="F219" s="1">
         <v>45963</v>
       </c>
       <c r="G219" t="s">
@@ -16778,7 +16876,7 @@
       <c r="E220" t="s">
         <v>29</v>
       </c>
-      <c r="F220" s="2">
+      <c r="F220" s="1">
         <v>45963</v>
       </c>
       <c r="G220" t="s">
@@ -16852,7 +16950,7 @@
       <c r="E221" t="s">
         <v>29</v>
       </c>
-      <c r="F221" s="2">
+      <c r="F221" s="1">
         <v>45963</v>
       </c>
       <c r="G221" t="s">
@@ -16929,7 +17027,7 @@
       <c r="E222" t="s">
         <v>29</v>
       </c>
-      <c r="F222" s="2">
+      <c r="F222" s="1">
         <v>45963</v>
       </c>
       <c r="G222" t="s">
@@ -17006,7 +17104,7 @@
       <c r="E223" t="s">
         <v>29</v>
       </c>
-      <c r="F223" s="2">
+      <c r="F223" s="1">
         <v>45963</v>
       </c>
       <c r="G223" t="s">
@@ -17080,7 +17178,7 @@
       <c r="E224" t="s">
         <v>29</v>
       </c>
-      <c r="F224" s="2">
+      <c r="F224" s="1">
         <v>45963</v>
       </c>
       <c r="G224" t="s">
@@ -17142,7 +17240,7 @@
       <c r="E225" t="s">
         <v>29</v>
       </c>
-      <c r="F225" s="2">
+      <c r="F225" s="1">
         <v>45963</v>
       </c>
       <c r="G225" t="s">
@@ -17216,7 +17314,7 @@
       <c r="E226" t="s">
         <v>403</v>
       </c>
-      <c r="F226" s="2">
+      <c r="F226" s="1">
         <v>45970</v>
       </c>
       <c r="G226" t="s">
@@ -17266,7 +17364,7 @@
       <c r="E227" t="s">
         <v>403</v>
       </c>
-      <c r="F227" s="2">
+      <c r="F227" s="1">
         <v>45970</v>
       </c>
       <c r="G227" t="s">
@@ -17316,7 +17414,7 @@
       <c r="E228" t="s">
         <v>403</v>
       </c>
-      <c r="F228" s="2">
+      <c r="F228" s="1">
         <v>45970</v>
       </c>
       <c r="G228" t="s">
@@ -17366,7 +17464,7 @@
       <c r="E229" t="s">
         <v>403</v>
       </c>
-      <c r="F229" s="2">
+      <c r="F229" s="1">
         <v>45970</v>
       </c>
       <c r="G229" t="s">
@@ -17419,7 +17517,7 @@
       <c r="E230" t="s">
         <v>403</v>
       </c>
-      <c r="F230" s="2">
+      <c r="F230" s="1">
         <v>45970</v>
       </c>
       <c r="G230" t="s">
@@ -17484,7 +17582,7 @@
       <c r="E231" t="s">
         <v>403</v>
       </c>
-      <c r="F231" s="2">
+      <c r="F231" s="1">
         <v>45970</v>
       </c>
       <c r="G231" t="s">
@@ -17555,7 +17653,7 @@
       <c r="E232" t="s">
         <v>403</v>
       </c>
-      <c r="F232" s="2">
+      <c r="F232" s="1">
         <v>45970</v>
       </c>
       <c r="G232" t="s">
@@ -17605,7 +17703,7 @@
       <c r="E233" t="s">
         <v>403</v>
       </c>
-      <c r="F233" s="2">
+      <c r="F233" s="1">
         <v>45970</v>
       </c>
       <c r="G233" t="s">
@@ -17655,7 +17753,7 @@
       <c r="E234" t="s">
         <v>403</v>
       </c>
-      <c r="F234" s="2">
+      <c r="F234" s="1">
         <v>45970</v>
       </c>
       <c r="G234" t="s">
@@ -17708,7 +17806,7 @@
       <c r="E235" t="s">
         <v>642</v>
       </c>
-      <c r="F235" s="2">
+      <c r="F235" s="1">
         <v>45991</v>
       </c>
       <c r="G235" t="s">
@@ -17782,7 +17880,7 @@
       <c r="E236" t="s">
         <v>642</v>
       </c>
-      <c r="F236" s="2">
+      <c r="F236" s="1">
         <v>45991</v>
       </c>
       <c r="G236" t="s">
@@ -17859,7 +17957,7 @@
       <c r="E237" t="s">
         <v>642</v>
       </c>
-      <c r="F237" s="2">
+      <c r="F237" s="1">
         <v>45991</v>
       </c>
       <c r="G237" t="s">
@@ -17936,7 +18034,7 @@
       <c r="E238" t="s">
         <v>642</v>
       </c>
-      <c r="F238" s="2">
+      <c r="F238" s="1">
         <v>45991</v>
       </c>
       <c r="G238" t="s">
@@ -18013,7 +18111,7 @@
       <c r="E239" t="s">
         <v>642</v>
       </c>
-      <c r="F239" s="2">
+      <c r="F239" s="1">
         <v>45991</v>
       </c>
       <c r="G239" t="s">
@@ -18090,7 +18188,7 @@
       <c r="E240" t="s">
         <v>642</v>
       </c>
-      <c r="F240" s="2">
+      <c r="F240" s="1">
         <v>45991</v>
       </c>
       <c r="G240" t="s">
@@ -18167,7 +18265,7 @@
       <c r="E241" t="s">
         <v>642</v>
       </c>
-      <c r="F241" s="2">
+      <c r="F241" s="1">
         <v>45991</v>
       </c>
       <c r="G241" t="s">
@@ -18244,7 +18342,7 @@
       <c r="E242" t="s">
         <v>642</v>
       </c>
-      <c r="F242" s="2">
+      <c r="F242" s="1">
         <v>45991</v>
       </c>
       <c r="G242" t="s">
@@ -18321,7 +18419,7 @@
       <c r="E243" t="s">
         <v>642</v>
       </c>
-      <c r="F243" s="2">
+      <c r="F243" s="1">
         <v>45991</v>
       </c>
       <c r="G243" t="s">
@@ -18398,7 +18496,7 @@
       <c r="E244" t="s">
         <v>642</v>
       </c>
-      <c r="F244" s="2">
+      <c r="F244" s="1">
         <v>45991</v>
       </c>
       <c r="G244" t="s">
@@ -18475,7 +18573,7 @@
       <c r="E245" t="s">
         <v>642</v>
       </c>
-      <c r="F245" s="2">
+      <c r="F245" s="1">
         <v>45991</v>
       </c>
       <c r="G245" t="s">
@@ -18552,7 +18650,7 @@
       <c r="E246" t="s">
         <v>642</v>
       </c>
-      <c r="F246" s="2">
+      <c r="F246" s="1">
         <v>45991</v>
       </c>
       <c r="G246" t="s">
@@ -18629,7 +18727,7 @@
       <c r="E247" t="s">
         <v>642</v>
       </c>
-      <c r="F247" s="2">
+      <c r="F247" s="1">
         <v>45991</v>
       </c>
       <c r="G247" t="s">
@@ -18706,7 +18804,7 @@
       <c r="E248" t="s">
         <v>642</v>
       </c>
-      <c r="F248" s="2">
+      <c r="F248" s="1">
         <v>45991</v>
       </c>
       <c r="G248" t="s">
@@ -18783,7 +18881,7 @@
       <c r="E249" t="s">
         <v>642</v>
       </c>
-      <c r="F249" s="2">
+      <c r="F249" s="1">
         <v>45991</v>
       </c>
       <c r="G249" t="s">
@@ -18860,7 +18958,7 @@
       <c r="E250" t="s">
         <v>642</v>
       </c>
-      <c r="F250" s="2">
+      <c r="F250" s="1">
         <v>45991</v>
       </c>
       <c r="G250" t="s">
@@ -18937,7 +19035,7 @@
       <c r="E251" t="s">
         <v>642</v>
       </c>
-      <c r="F251" s="2">
+      <c r="F251" s="1">
         <v>45991</v>
       </c>
       <c r="G251" t="s">
@@ -19014,7 +19112,7 @@
       <c r="E252" t="s">
         <v>642</v>
       </c>
-      <c r="F252" s="2">
+      <c r="F252" s="1">
         <v>45991</v>
       </c>
       <c r="G252" t="s">
@@ -19091,7 +19189,7 @@
       <c r="E253" t="s">
         <v>922</v>
       </c>
-      <c r="F253" s="2">
+      <c r="F253" s="1">
         <v>46012</v>
       </c>
       <c r="G253" t="s">
@@ -19168,7 +19266,7 @@
       <c r="E254" t="s">
         <v>922</v>
       </c>
-      <c r="F254" s="2">
+      <c r="F254" s="1">
         <v>46012</v>
       </c>
       <c r="G254" t="s">
@@ -19245,7 +19343,7 @@
       <c r="E255" t="s">
         <v>922</v>
       </c>
-      <c r="F255" s="2">
+      <c r="F255" s="1">
         <v>46012</v>
       </c>
       <c r="G255" t="s">
@@ -19322,7 +19420,7 @@
       <c r="E256" t="s">
         <v>922</v>
       </c>
-      <c r="F256" s="2">
+      <c r="F256" s="1">
         <v>46012</v>
       </c>
       <c r="G256" t="s">
@@ -19396,7 +19494,7 @@
       <c r="E257" t="s">
         <v>922</v>
       </c>
-      <c r="F257" s="2">
+      <c r="F257" s="1">
         <v>46012</v>
       </c>
       <c r="G257" t="s">
@@ -19473,7 +19571,7 @@
       <c r="E258" t="s">
         <v>922</v>
       </c>
-      <c r="F258" s="2">
+      <c r="F258" s="1">
         <v>46012</v>
       </c>
       <c r="G258" t="s">
@@ -19550,7 +19648,7 @@
       <c r="E259" t="s">
         <v>922</v>
       </c>
-      <c r="F259" s="2">
+      <c r="F259" s="1">
         <v>46012</v>
       </c>
       <c r="G259" t="s">
@@ -19627,7 +19725,7 @@
       <c r="E260" t="s">
         <v>922</v>
       </c>
-      <c r="F260" s="2">
+      <c r="F260" s="1">
         <v>46012</v>
       </c>
       <c r="G260" t="s">
@@ -19704,7 +19802,7 @@
       <c r="E261" t="s">
         <v>922</v>
       </c>
-      <c r="F261" s="2">
+      <c r="F261" s="1">
         <v>46012</v>
       </c>
       <c r="G261" t="s">
@@ -19781,7 +19879,7 @@
       <c r="E262" t="s">
         <v>922</v>
       </c>
-      <c r="F262" s="2">
+      <c r="F262" s="1">
         <v>46012</v>
       </c>
       <c r="G262" t="s">
@@ -19858,7 +19956,7 @@
       <c r="E263" t="s">
         <v>922</v>
       </c>
-      <c r="F263" s="2">
+      <c r="F263" s="1">
         <v>46012</v>
       </c>
       <c r="G263" t="s">
@@ -19935,7 +20033,7 @@
       <c r="E264" t="s">
         <v>922</v>
       </c>
-      <c r="F264" s="2">
+      <c r="F264" s="1">
         <v>46012</v>
       </c>
       <c r="G264" t="s">
@@ -20012,7 +20110,7 @@
       <c r="E265" t="s">
         <v>922</v>
       </c>
-      <c r="F265" s="2">
+      <c r="F265" s="1">
         <v>46012</v>
       </c>
       <c r="G265" t="s">
@@ -20089,7 +20187,7 @@
       <c r="E266" t="s">
         <v>922</v>
       </c>
-      <c r="F266" s="2">
+      <c r="F266" s="1">
         <v>46012</v>
       </c>
       <c r="G266" t="s">
@@ -20166,7 +20264,7 @@
       <c r="E267" t="s">
         <v>922</v>
       </c>
-      <c r="F267" s="2">
+      <c r="F267" s="1">
         <v>46012</v>
       </c>
       <c r="G267" t="s">
@@ -20243,7 +20341,7 @@
       <c r="E268" t="s">
         <v>922</v>
       </c>
-      <c r="F268" s="2">
+      <c r="F268" s="1">
         <v>46012</v>
       </c>
       <c r="G268" t="s">
@@ -20320,7 +20418,7 @@
       <c r="E269" t="s">
         <v>922</v>
       </c>
-      <c r="F269" s="2">
+      <c r="F269" s="1">
         <v>46012</v>
       </c>
       <c r="G269" t="s">
@@ -20397,7 +20495,7 @@
       <c r="E270" t="s">
         <v>922</v>
       </c>
-      <c r="F270" s="2">
+      <c r="F270" s="1">
         <v>46012</v>
       </c>
       <c r="G270" t="s">
@@ -20474,7 +20572,7 @@
       <c r="E271" t="s">
         <v>403</v>
       </c>
-      <c r="F271" s="2">
+      <c r="F271" s="1">
         <v>46040</v>
       </c>
       <c r="G271" t="s">
@@ -20539,7 +20637,7 @@
       <c r="E272" t="s">
         <v>403</v>
       </c>
-      <c r="F272" s="2">
+      <c r="F272" s="1">
         <v>46040</v>
       </c>
       <c r="G272" t="s">
@@ -20604,7 +20702,7 @@
       <c r="E273" t="s">
         <v>403</v>
       </c>
-      <c r="F273" s="2">
+      <c r="F273" s="1">
         <v>46040</v>
       </c>
       <c r="G273" t="s">
@@ -20669,7 +20767,7 @@
       <c r="E274" t="s">
         <v>403</v>
       </c>
-      <c r="F274" s="2">
+      <c r="F274" s="1">
         <v>46040</v>
       </c>
       <c r="G274" t="s">
@@ -20734,7 +20832,7 @@
       <c r="E275" t="s">
         <v>403</v>
       </c>
-      <c r="F275" s="2">
+      <c r="F275" s="1">
         <v>46040</v>
       </c>
       <c r="G275" t="s">
@@ -20799,7 +20897,7 @@
       <c r="E276" t="s">
         <v>403</v>
       </c>
-      <c r="F276" s="2">
+      <c r="F276" s="1">
         <v>46040</v>
       </c>
       <c r="G276" t="s">
@@ -20864,7 +20962,7 @@
       <c r="E277" t="s">
         <v>403</v>
       </c>
-      <c r="F277" s="2">
+      <c r="F277" s="1">
         <v>46040</v>
       </c>
       <c r="G277" t="s">
@@ -20929,7 +21027,7 @@
       <c r="E278" t="s">
         <v>403</v>
       </c>
-      <c r="F278" s="2">
+      <c r="F278" s="1">
         <v>46040</v>
       </c>
       <c r="G278" t="s">
@@ -20994,7 +21092,7 @@
       <c r="E279" t="s">
         <v>403</v>
       </c>
-      <c r="F279" s="2">
+      <c r="F279" s="1">
         <v>46040</v>
       </c>
       <c r="G279" t="s">
@@ -21059,7 +21157,7 @@
       <c r="E280" t="s">
         <v>403</v>
       </c>
-      <c r="F280" s="2">
+      <c r="F280" s="1">
         <v>46040</v>
       </c>
       <c r="G280" t="s">
@@ -21124,7 +21222,7 @@
       <c r="E281" t="s">
         <v>403</v>
       </c>
-      <c r="F281" s="2">
+      <c r="F281" s="1">
         <v>46040</v>
       </c>
       <c r="G281" t="s">
@@ -21189,7 +21287,7 @@
       <c r="E282" t="s">
         <v>403</v>
       </c>
-      <c r="F282" s="2">
+      <c r="F282" s="1">
         <v>46040</v>
       </c>
       <c r="G282" t="s">
@@ -21254,7 +21352,7 @@
       <c r="E283" t="s">
         <v>403</v>
       </c>
-      <c r="F283" s="2">
+      <c r="F283" s="1">
         <v>46040</v>
       </c>
       <c r="G283" t="s">
@@ -21319,7 +21417,7 @@
       <c r="E284" t="s">
         <v>403</v>
       </c>
-      <c r="F284" s="2">
+      <c r="F284" s="1">
         <v>46040</v>
       </c>
       <c r="G284" t="s">
@@ -21384,7 +21482,7 @@
       <c r="E285" t="s">
         <v>403</v>
       </c>
-      <c r="F285" s="2">
+      <c r="F285" s="1">
         <v>46040</v>
       </c>
       <c r="G285" t="s">
@@ -21458,7 +21556,7 @@
       <c r="E286" t="s">
         <v>403</v>
       </c>
-      <c r="F286" s="2">
+      <c r="F286" s="1">
         <v>46040</v>
       </c>
       <c r="G286" t="s">
@@ -21523,7 +21621,7 @@
       <c r="E287" t="s">
         <v>403</v>
       </c>
-      <c r="F287" s="2">
+      <c r="F287" s="1">
         <v>46040</v>
       </c>
       <c r="G287" t="s">
@@ -21588,7 +21686,7 @@
       <c r="E288" t="s">
         <v>403</v>
       </c>
-      <c r="F288" s="2">
+      <c r="F288" s="1">
         <v>46040</v>
       </c>
       <c r="G288" t="s">
@@ -21653,7 +21751,7 @@
       <c r="E289" t="s">
         <v>403</v>
       </c>
-      <c r="F289" s="2">
+      <c r="F289" s="1">
         <v>46040</v>
       </c>
       <c r="G289" t="s">
@@ -21718,7 +21816,7 @@
       <c r="E290" t="s">
         <v>403</v>
       </c>
-      <c r="F290" s="2">
+      <c r="F290" s="1">
         <v>46040</v>
       </c>
       <c r="G290" t="s">
@@ -21783,7 +21881,7 @@
       <c r="E291" t="s">
         <v>403</v>
       </c>
-      <c r="F291" s="2">
+      <c r="F291" s="1">
         <v>46040</v>
       </c>
       <c r="G291" t="s">
@@ -21848,7 +21946,7 @@
       <c r="E292" t="s">
         <v>403</v>
       </c>
-      <c r="F292" s="2">
+      <c r="F292" s="1">
         <v>46040</v>
       </c>
       <c r="G292" t="s">
@@ -21913,7 +22011,7 @@
       <c r="E293" t="s">
         <v>403</v>
       </c>
-      <c r="F293" s="2">
+      <c r="F293" s="1">
         <v>46040</v>
       </c>
       <c r="G293" t="s">
@@ -21978,7 +22076,7 @@
       <c r="E294" t="s">
         <v>403</v>
       </c>
-      <c r="F294" s="2">
+      <c r="F294" s="1">
         <v>46040</v>
       </c>
       <c r="G294" t="s">
@@ -22043,7 +22141,7 @@
       <c r="E295" t="s">
         <v>403</v>
       </c>
-      <c r="F295" s="2">
+      <c r="F295" s="1">
         <v>46040</v>
       </c>
       <c r="G295" t="s">
@@ -22108,7 +22206,7 @@
       <c r="E296" t="s">
         <v>403</v>
       </c>
-      <c r="F296" s="2">
+      <c r="F296" s="1">
         <v>46040</v>
       </c>
       <c r="G296" t="s">
@@ -22173,7 +22271,7 @@
       <c r="E297" t="s">
         <v>403</v>
       </c>
-      <c r="F297" s="2">
+      <c r="F297" s="1">
         <v>46040</v>
       </c>
       <c r="G297" t="s">
@@ -22238,7 +22336,7 @@
       <c r="E298" t="s">
         <v>403</v>
       </c>
-      <c r="F298" s="2">
+      <c r="F298" s="1">
         <v>46040</v>
       </c>
       <c r="G298" t="s">
@@ -22303,7 +22401,7 @@
       <c r="E299" t="s">
         <v>403</v>
       </c>
-      <c r="F299" s="2">
+      <c r="F299" s="1">
         <v>46040</v>
       </c>
       <c r="G299" t="s">
@@ -22368,7 +22466,7 @@
       <c r="E300" t="s">
         <v>403</v>
       </c>
-      <c r="F300" s="2">
+      <c r="F300" s="1">
         <v>46040</v>
       </c>
       <c r="G300" t="s">
@@ -22433,7 +22531,7 @@
       <c r="E301" t="s">
         <v>403</v>
       </c>
-      <c r="F301" s="2">
+      <c r="F301" s="1">
         <v>46040</v>
       </c>
       <c r="G301" t="s">
@@ -22498,7 +22596,7 @@
       <c r="E302" t="s">
         <v>403</v>
       </c>
-      <c r="F302" s="2">
+      <c r="F302" s="1">
         <v>46040</v>
       </c>
       <c r="G302" t="s">
@@ -22563,7 +22661,7 @@
       <c r="E303" t="s">
         <v>29</v>
       </c>
-      <c r="F303" s="2">
+      <c r="F303" s="1">
         <v>46047</v>
       </c>
       <c r="G303" t="s">
@@ -22640,7 +22738,7 @@
       <c r="E304" t="s">
         <v>29</v>
       </c>
-      <c r="F304" s="2">
+      <c r="F304" s="1">
         <v>46047</v>
       </c>
       <c r="G304" t="s">
@@ -22717,7 +22815,7 @@
       <c r="E305" t="s">
         <v>29</v>
       </c>
-      <c r="F305" s="2">
+      <c r="F305" s="1">
         <v>46047</v>
       </c>
       <c r="G305" t="s">
@@ -22782,7 +22880,7 @@
       <c r="E306" t="s">
         <v>29</v>
       </c>
-      <c r="F306" s="2">
+      <c r="F306" s="1">
         <v>46047</v>
       </c>
       <c r="G306" t="s">
@@ -22847,7 +22945,7 @@
       <c r="E307" t="s">
         <v>29</v>
       </c>
-      <c r="F307" s="2">
+      <c r="F307" s="1">
         <v>46047</v>
       </c>
       <c r="G307" t="s">
@@ -22912,7 +23010,7 @@
       <c r="E308" t="s">
         <v>29</v>
       </c>
-      <c r="F308" s="2">
+      <c r="F308" s="1">
         <v>46047</v>
       </c>
       <c r="G308" t="s">
@@ -22986,7 +23084,7 @@
       <c r="E309" t="s">
         <v>29</v>
       </c>
-      <c r="F309" s="2">
+      <c r="F309" s="1">
         <v>46047</v>
       </c>
       <c r="G309" t="s">
@@ -23063,7 +23161,7 @@
       <c r="E310" t="s">
         <v>29</v>
       </c>
-      <c r="F310" s="2">
+      <c r="F310" s="1">
         <v>46047</v>
       </c>
       <c r="G310" t="s">
@@ -23140,7 +23238,7 @@
       <c r="E311" t="s">
         <v>29</v>
       </c>
-      <c r="F311" s="2">
+      <c r="F311" s="1">
         <v>46047</v>
       </c>
       <c r="G311" t="s">
@@ -23217,7 +23315,7 @@
       <c r="E312" t="s">
         <v>29</v>
       </c>
-      <c r="F312" s="2">
+      <c r="F312" s="1">
         <v>46047</v>
       </c>
       <c r="G312" t="s">
@@ -23294,7 +23392,7 @@
       <c r="E313" t="s">
         <v>29</v>
       </c>
-      <c r="F313" s="2">
+      <c r="F313" s="1">
         <v>46047</v>
       </c>
       <c r="G313" t="s">
@@ -23371,7 +23469,7 @@
       <c r="E314" t="s">
         <v>29</v>
       </c>
-      <c r="F314" s="2">
+      <c r="F314" s="1">
         <v>46047</v>
       </c>
       <c r="G314" t="s">
@@ -23434,5 +23532,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>